<commit_message>
Add product category filter
</commit_message>
<xml_diff>
--- a/Products.xlsx
+++ b/Products.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="58">
   <si>
     <t>id</t>
   </si>
@@ -58,6 +58,9 @@
     <t>size</t>
   </si>
   <si>
+    <t>Category</t>
+  </si>
+  <si>
     <t>VR</t>
   </si>
   <si>
@@ -73,6 +76,9 @@
     <t>1*1</t>
   </si>
   <si>
+    <t>Play</t>
+  </si>
+  <si>
     <t>GP</t>
   </si>
   <si>
@@ -85,6 +91,9 @@
     <t>1*2</t>
   </si>
   <si>
+    <t>Electronic</t>
+  </si>
+  <si>
     <t>SF</t>
   </si>
   <si>
@@ -121,6 +130,9 @@
     <t>1*5</t>
   </si>
   <si>
+    <t>Decoration</t>
+  </si>
+  <si>
     <t>BATHROOM_SETS</t>
   </si>
   <si>
@@ -133,6 +145,9 @@
     <t>1*6</t>
   </si>
   <si>
+    <t>Life</t>
+  </si>
+  <si>
     <t>COFFEE_MAKER</t>
   </si>
   <si>
@@ -145,6 +160,9 @@
     <t>1*7</t>
   </si>
   <si>
+    <t>Food</t>
+  </si>
+  <si>
     <t>SNACK_BOX</t>
   </si>
   <si>
@@ -169,6 +187,9 @@
     <t>1*9</t>
   </si>
   <si>
+    <t>Bake</t>
+  </si>
+  <si>
     <t>STORGE_BOX</t>
   </si>
   <si>
@@ -179,6 +200,9 @@
   </si>
   <si>
     <t>1*10</t>
+  </si>
+  <si>
+    <t>Storge</t>
   </si>
 </sst>
 </file>
@@ -1112,7 +1136,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.1"/>
   <cols>
     <col min="1" max="1" width="14.6576576576577" customWidth="1"/>
@@ -1121,9 +1145,10 @@
     <col min="4" max="4" width="29.4954954954955" customWidth="1"/>
     <col min="5" max="5" width="32.4324324324324" customWidth="1"/>
     <col min="7" max="7" width="13.8918918918919" customWidth="1"/>
+    <col min="10" max="10" width="15.2612612612613" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:10">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1151,295 +1176,328 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" ht="14.15" spans="1:9">
+    <row r="2" ht="14.15" spans="1:10">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" s="1">
         <v>500</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H2">
         <v>2</v>
       </c>
       <c r="I2" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="J2" t="s">
+        <v>15</v>
       </c>
     </row>
-    <row r="3" ht="14.15" spans="1:9">
+    <row r="3" ht="14.15" spans="1:10">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C3" s="1">
         <v>1000</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F3">
         <v>2</v>
       </c>
       <c r="G3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H3">
         <v>3</v>
       </c>
       <c r="I3" t="s">
-        <v>17</v>
+        <v>19</v>
+      </c>
+      <c r="J3" t="s">
+        <v>20</v>
       </c>
     </row>
-    <row r="4" ht="14.15" spans="1:9">
+    <row r="4" ht="14.15" spans="1:10">
       <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C4" s="1">
         <v>520</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F4">
         <v>3</v>
       </c>
       <c r="G4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H4">
         <v>4</v>
       </c>
       <c r="I4" t="s">
-        <v>21</v>
+        <v>24</v>
+      </c>
+      <c r="J4" t="s">
+        <v>20</v>
       </c>
     </row>
-    <row r="5" ht="14.15" spans="1:9">
+    <row r="5" ht="14.15" spans="1:10">
       <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C5" s="1">
         <v>1314</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F5">
         <v>4</v>
       </c>
       <c r="G5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H5">
         <v>5</v>
       </c>
       <c r="I5" t="s">
-        <v>25</v>
+        <v>28</v>
+      </c>
+      <c r="J5" t="s">
+        <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:10">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C6">
         <v>9999</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F6">
         <v>5</v>
       </c>
       <c r="G6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H6">
         <v>6</v>
       </c>
       <c r="I6" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="J6" t="s">
+        <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:10">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C7">
         <v>8888</v>
       </c>
       <c r="D7" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E7" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="F7">
         <v>6</v>
       </c>
       <c r="G7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H7">
         <v>7</v>
       </c>
       <c r="I7" t="s">
-        <v>33</v>
+        <v>37</v>
+      </c>
+      <c r="J7" t="s">
+        <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:10">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="C8">
         <v>6666</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="F8">
         <v>7</v>
       </c>
       <c r="G8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H8">
         <v>8</v>
       </c>
       <c r="I8" t="s">
-        <v>37</v>
+        <v>42</v>
+      </c>
+      <c r="J8" t="s">
+        <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:10">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="C9">
         <v>4444</v>
       </c>
       <c r="D9" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="E9" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="F9">
         <v>8</v>
       </c>
       <c r="G9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H9">
         <v>9</v>
       </c>
       <c r="I9" t="s">
-        <v>41</v>
+        <v>47</v>
+      </c>
+      <c r="J9" t="s">
+        <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:10">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="C10">
         <v>2222</v>
       </c>
       <c r="D10" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="E10" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="F10">
         <v>9</v>
       </c>
       <c r="G10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H10">
         <v>10</v>
       </c>
       <c r="I10" t="s">
-        <v>45</v>
+        <v>51</v>
+      </c>
+      <c r="J10" t="s">
+        <v>52</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:10">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C11">
         <v>1111</v>
       </c>
       <c r="D11" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="E11" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F11">
         <v>10</v>
       </c>
       <c r="G11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H11">
         <v>11</v>
       </c>
       <c r="I11" t="s">
-        <v>49</v>
+        <v>56</v>
+      </c>
+      <c r="J11" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Decoration and Food categories
</commit_message>
<xml_diff>
--- a/Products.xlsx
+++ b/Products.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="57">
   <si>
     <t>id</t>
   </si>
@@ -76,7 +76,7 @@
     <t>1*1</t>
   </si>
   <si>
-    <t>Play</t>
+    <t>Electronics</t>
   </si>
   <si>
     <t>GP</t>
@@ -91,9 +91,6 @@
     <t>1*2</t>
   </si>
   <si>
-    <t>Electronic</t>
-  </si>
-  <si>
     <t>SF</t>
   </si>
   <si>
@@ -145,7 +142,7 @@
     <t>1*6</t>
   </si>
   <si>
-    <t>Life</t>
+    <t>Storage</t>
   </si>
   <si>
     <t>COFFEE_MAKER</t>
@@ -160,21 +157,24 @@
     <t>1*7</t>
   </si>
   <si>
+    <t>Coffee</t>
+  </si>
+  <si>
+    <t>SNACK_BOX</t>
+  </si>
+  <si>
+    <t>WE WILL BE TOGETHER FOREVER</t>
+  </si>
+  <si>
+    <t>/static/image/SNACK_BOX.png</t>
+  </si>
+  <si>
+    <t>1*8</t>
+  </si>
+  <si>
     <t>Food</t>
   </si>
   <si>
-    <t>SNACK_BOX</t>
-  </si>
-  <si>
-    <t>WE WILL BE TOGETHER FOREVER</t>
-  </si>
-  <si>
-    <t>/static/image/SNACK_BOX.png</t>
-  </si>
-  <si>
-    <t>1*8</t>
-  </si>
-  <si>
     <t>BAKE_SET</t>
   </si>
   <si>
@@ -187,7 +187,7 @@
     <t>1*9</t>
   </si>
   <si>
-    <t>Bake</t>
+    <t>Bakeware</t>
   </si>
   <si>
     <t>STORGE_BOX</t>
@@ -200,9 +200,6 @@
   </si>
   <si>
     <t>1*10</t>
-  </si>
-  <si>
-    <t>Storge</t>
   </si>
 </sst>
 </file>
@@ -215,13 +212,19 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+      <color rgb="FFA5D6FF"/>
+      <name val="Consolas"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -688,141 +691,144 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1208,7 +1214,7 @@
       <c r="I2" t="s">
         <v>14</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="2" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1240,8 +1246,8 @@
       <c r="I3" t="s">
         <v>19</v>
       </c>
-      <c r="J3" t="s">
-        <v>20</v>
+      <c r="J3" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="4" ht="14.15" spans="1:10">
@@ -1249,16 +1255,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C4" s="1">
         <v>520</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="F4">
         <v>3</v>
@@ -1270,10 +1276,10 @@
         <v>4</v>
       </c>
       <c r="I4" t="s">
-        <v>24</v>
-      </c>
-      <c r="J4" t="s">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="5" ht="14.15" spans="1:10">
@@ -1281,16 +1287,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5" s="1">
         <v>1314</v>
       </c>
       <c r="D5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="F5">
         <v>4</v>
@@ -1302,10 +1308,10 @@
         <v>5</v>
       </c>
       <c r="I5" t="s">
-        <v>28</v>
-      </c>
-      <c r="J5" t="s">
-        <v>20</v>
+        <v>27</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -1313,16 +1319,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C6">
         <v>9999</v>
       </c>
       <c r="D6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" t="s">
         <v>30</v>
-      </c>
-      <c r="E6" t="s">
-        <v>31</v>
       </c>
       <c r="F6">
         <v>5</v>
@@ -1334,10 +1340,10 @@
         <v>6</v>
       </c>
       <c r="I6" t="s">
+        <v>31</v>
+      </c>
+      <c r="J6" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="J6" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -1345,16 +1351,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C7">
         <v>8888</v>
       </c>
       <c r="D7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" t="s">
         <v>35</v>
-      </c>
-      <c r="E7" t="s">
-        <v>36</v>
       </c>
       <c r="F7">
         <v>6</v>
@@ -1366,10 +1372,10 @@
         <v>7</v>
       </c>
       <c r="I7" t="s">
+        <v>36</v>
+      </c>
+      <c r="J7" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="J7" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -1377,16 +1383,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C8">
         <v>6666</v>
       </c>
       <c r="D8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" t="s">
         <v>40</v>
-      </c>
-      <c r="E8" t="s">
-        <v>41</v>
       </c>
       <c r="F8">
         <v>7</v>
@@ -1398,10 +1404,10 @@
         <v>8</v>
       </c>
       <c r="I8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J8" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="J8" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -1409,16 +1415,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C9">
         <v>4444</v>
       </c>
       <c r="D9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E9" t="s">
         <v>45</v>
-      </c>
-      <c r="E9" t="s">
-        <v>46</v>
       </c>
       <c r="F9">
         <v>8</v>
@@ -1430,10 +1436,10 @@
         <v>9</v>
       </c>
       <c r="I9" t="s">
+        <v>46</v>
+      </c>
+      <c r="J9" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="J9" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -1464,7 +1470,7 @@
       <c r="I10" t="s">
         <v>51</v>
       </c>
-      <c r="J10" t="s">
+      <c r="J10" s="2" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1496,8 +1502,8 @@
       <c r="I11" t="s">
         <v>56</v>
       </c>
-      <c r="J11" t="s">
-        <v>57</v>
+      <c r="J11" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add product gallery images and video
</commit_message>
<xml_diff>
--- a/Products.xlsx
+++ b/Products.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="74">
   <si>
     <t>id</t>
   </si>
@@ -46,6 +46,24 @@
     <t>image</t>
   </si>
   <si>
+    <t>image_2</t>
+  </si>
+  <si>
+    <t>image_3</t>
+  </si>
+  <si>
+    <t>image_4</t>
+  </si>
+  <si>
+    <t>image_5</t>
+  </si>
+  <si>
+    <t>image_6</t>
+  </si>
+  <si>
+    <t>video</t>
+  </si>
+  <si>
     <t>moq</t>
   </si>
   <si>
@@ -83,6 +101,24 @@
   </si>
   <si>
     <t>/static/image/VR.jpg</t>
+  </si>
+  <si>
+    <t>/static/image/row_salmon.jpg</t>
+  </si>
+  <si>
+    <t>/static/image/salmon.jpg</t>
+  </si>
+  <si>
+    <t>/static/image/set.jpg</t>
+  </si>
+  <si>
+    <t>/static/image/sp.jpg</t>
+  </si>
+  <si>
+    <t>/static/image/steak.jpg</t>
+  </si>
+  <si>
+    <t>/static/video/sp2.mp4</t>
   </si>
   <si>
     <t>PP</t>
@@ -836,8 +872,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1157,7 +1196,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.1"/>
   <cols>
     <col min="1" max="1" width="14.6576576576577" customWidth="1"/>
@@ -1165,16 +1204,22 @@
     <col min="3" max="3" width="14.7387387387387" customWidth="1"/>
     <col min="4" max="4" width="29.4954954954955" customWidth="1"/>
     <col min="5" max="5" width="32.4324324324324" customWidth="1"/>
-    <col min="7" max="7" width="13.8918918918919" customWidth="1"/>
-    <col min="10" max="10" width="15.2612612612613" customWidth="1"/>
-    <col min="11" max="11" width="11.1711711711712" customWidth="1"/>
-    <col min="12" max="12" width="11.6216216216216" customWidth="1"/>
-    <col min="13" max="13" width="11.3513513513514" customWidth="1"/>
-    <col min="14" max="14" width="11.7117117117117" customWidth="1"/>
-    <col min="15" max="15" width="13.3513513513514" customWidth="1"/>
+    <col min="6" max="6" width="29.4324324324324" customWidth="1"/>
+    <col min="7" max="7" width="25.7927927927928" customWidth="1"/>
+    <col min="8" max="8" width="22.8828828828829" customWidth="1"/>
+    <col min="9" max="9" width="20.981981981982" customWidth="1"/>
+    <col min="10" max="10" width="24.4324324324324" customWidth="1"/>
+    <col min="11" max="11" width="28.2432432432432" customWidth="1"/>
+    <col min="13" max="13" width="13.8918918918919" customWidth="1"/>
+    <col min="16" max="16" width="15.2612612612613" customWidth="1"/>
+    <col min="17" max="17" width="11.1711711711712" customWidth="1"/>
+    <col min="18" max="18" width="11.6216216216216" customWidth="1"/>
+    <col min="19" max="19" width="11.3513513513514" customWidth="1"/>
+    <col min="20" max="20" width="11.7117117117117" customWidth="1"/>
+    <col min="21" max="21" width="13.3513513513514" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:21">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1190,13 +1235,13 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="I1" t="s">
@@ -1205,7 +1250,7 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
       <c r="L1" t="s">
@@ -1220,474 +1265,510 @@
       <c r="O1" t="s">
         <v>14</v>
       </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="2" ht="14.15" spans="1:15">
-      <c r="A2" s="1">
+    <row r="2" ht="14.15" spans="1:21">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="1">
+      <c r="B2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="2">
         <v>500</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2">
+      <c r="D2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" t="s">
+        <v>25</v>
+      </c>
+      <c r="H2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2" t="s">
+        <v>28</v>
+      </c>
+      <c r="K2" t="s">
+        <v>29</v>
+      </c>
+      <c r="L2">
         <v>500</v>
       </c>
-      <c r="G2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H2">
-        <v>2</v>
-      </c>
-      <c r="I2" t="s">
-        <v>19</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2">
-        <v>5</v>
-      </c>
-      <c r="L2">
-        <v>4</v>
-      </c>
-      <c r="M2">
-        <v>3</v>
+      <c r="M2" t="s">
+        <v>30</v>
       </c>
       <c r="N2">
         <v>2</v>
       </c>
-      <c r="O2">
+      <c r="O2" t="s">
+        <v>31</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q2">
+        <v>5</v>
+      </c>
+      <c r="R2">
+        <v>4</v>
+      </c>
+      <c r="S2">
+        <v>3</v>
+      </c>
+      <c r="T2">
+        <v>2</v>
+      </c>
+      <c r="U2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" ht="14.15" spans="1:15">
-      <c r="A3" s="1">
+    <row r="3" ht="14.15" spans="1:21">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" s="1">
+      <c r="B3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="2">
         <v>1000</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3">
+      <c r="D3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="L3">
         <v>500</v>
       </c>
-      <c r="G3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3">
+      <c r="M3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N3">
         <v>3</v>
       </c>
-      <c r="I3" t="s">
-        <v>24</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3">
+      <c r="O3" t="s">
+        <v>36</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q3">
         <v>5</v>
       </c>
-      <c r="L3">
+      <c r="R3">
         <v>4</v>
       </c>
-      <c r="M3">
+      <c r="S3">
         <v>3</v>
       </c>
-      <c r="N3">
+      <c r="T3">
         <v>2</v>
       </c>
-      <c r="O3">
+      <c r="U3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" ht="14.15" spans="1:15">
-      <c r="A4" s="1">
+    <row r="4" ht="14.15" spans="1:21">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4" s="1">
+      <c r="B4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="2">
         <v>520</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4">
+      <c r="D4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="L4">
         <v>500</v>
       </c>
-      <c r="G4" t="s">
-        <v>18</v>
-      </c>
-      <c r="H4">
+      <c r="M4" t="s">
+        <v>30</v>
+      </c>
+      <c r="N4">
         <v>4</v>
       </c>
-      <c r="I4" t="s">
-        <v>28</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K4">
+      <c r="O4" t="s">
+        <v>40</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q4">
         <v>5</v>
       </c>
-      <c r="L4">
+      <c r="R4">
         <v>4</v>
       </c>
-      <c r="M4">
+      <c r="S4">
         <v>3</v>
       </c>
-      <c r="N4">
+      <c r="T4">
         <v>2</v>
       </c>
-      <c r="O4">
+      <c r="U4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" ht="14.15" spans="1:15">
-      <c r="A5" s="1">
+    <row r="5" ht="14.15" spans="1:21">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" s="1">
+      <c r="B5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="2">
         <v>1314</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L5">
+        <v>500</v>
+      </c>
+      <c r="M5" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5">
-        <v>500</v>
-      </c>
-      <c r="G5" t="s">
-        <v>18</v>
-      </c>
-      <c r="H5">
+      <c r="N5">
         <v>5</v>
       </c>
-      <c r="I5" t="s">
+      <c r="O5" t="s">
+        <v>44</v>
+      </c>
+      <c r="P5" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="J5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K5">
+      <c r="Q5">
         <v>5</v>
       </c>
-      <c r="L5">
+      <c r="R5">
         <v>4</v>
       </c>
-      <c r="M5">
+      <c r="S5">
         <v>3</v>
       </c>
-      <c r="N5">
+      <c r="T5">
         <v>2</v>
       </c>
-      <c r="O5">
+      <c r="U5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:21">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="C6">
         <v>9999</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E6" t="s">
-        <v>35</v>
-      </c>
-      <c r="F6">
+        <v>47</v>
+      </c>
+      <c r="L6">
         <v>500</v>
       </c>
-      <c r="G6" t="s">
-        <v>18</v>
-      </c>
-      <c r="H6">
+      <c r="M6" t="s">
+        <v>30</v>
+      </c>
+      <c r="N6">
         <v>6</v>
       </c>
-      <c r="I6" t="s">
-        <v>36</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="K6">
+      <c r="O6" t="s">
+        <v>48</v>
+      </c>
+      <c r="P6" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q6">
         <v>5</v>
       </c>
-      <c r="L6">
+      <c r="R6">
         <v>4</v>
       </c>
-      <c r="M6">
+      <c r="S6">
         <v>3</v>
       </c>
-      <c r="N6">
+      <c r="T6">
         <v>2</v>
       </c>
-      <c r="O6">
+      <c r="U6">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:21">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="C7">
         <v>8888</v>
       </c>
       <c r="D7" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
-      </c>
-      <c r="F7">
+        <v>52</v>
+      </c>
+      <c r="L7">
         <v>500</v>
       </c>
-      <c r="G7" t="s">
-        <v>18</v>
-      </c>
-      <c r="H7">
+      <c r="M7" t="s">
+        <v>30</v>
+      </c>
+      <c r="N7">
         <v>7</v>
       </c>
-      <c r="I7" t="s">
-        <v>41</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="K7">
+      <c r="O7" t="s">
+        <v>53</v>
+      </c>
+      <c r="P7" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q7">
         <v>5</v>
       </c>
-      <c r="L7">
+      <c r="R7">
         <v>4</v>
       </c>
-      <c r="M7">
+      <c r="S7">
         <v>3</v>
       </c>
-      <c r="N7">
+      <c r="T7">
         <v>2</v>
       </c>
-      <c r="O7">
+      <c r="U7">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:21">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="C8">
         <v>6666</v>
       </c>
       <c r="D8" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="E8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F8">
+        <v>57</v>
+      </c>
+      <c r="L8">
         <v>500</v>
       </c>
-      <c r="G8" t="s">
-        <v>18</v>
-      </c>
-      <c r="H8">
+      <c r="M8" t="s">
+        <v>30</v>
+      </c>
+      <c r="N8">
         <v>8</v>
       </c>
-      <c r="I8" t="s">
-        <v>46</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="K8">
+      <c r="O8" t="s">
+        <v>58</v>
+      </c>
+      <c r="P8" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q8">
         <v>5</v>
       </c>
-      <c r="L8">
+      <c r="R8">
         <v>4</v>
       </c>
-      <c r="M8">
+      <c r="S8">
         <v>3</v>
       </c>
-      <c r="N8">
+      <c r="T8">
         <v>2</v>
       </c>
-      <c r="O8">
+      <c r="U8">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:21">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="C9">
         <v>4444</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="E9" t="s">
-        <v>50</v>
-      </c>
-      <c r="F9">
+        <v>62</v>
+      </c>
+      <c r="L9">
         <v>500</v>
       </c>
-      <c r="G9" t="s">
-        <v>18</v>
-      </c>
-      <c r="H9">
+      <c r="M9" t="s">
+        <v>30</v>
+      </c>
+      <c r="N9">
         <v>9</v>
       </c>
-      <c r="I9" t="s">
-        <v>51</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="K9">
+      <c r="O9" t="s">
+        <v>63</v>
+      </c>
+      <c r="P9" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q9">
         <v>5</v>
       </c>
-      <c r="L9">
+      <c r="R9">
         <v>4</v>
       </c>
-      <c r="M9">
+      <c r="S9">
         <v>3</v>
       </c>
-      <c r="N9">
+      <c r="T9">
         <v>2</v>
       </c>
-      <c r="O9">
+      <c r="U9">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:21">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="C10">
         <v>2222</v>
       </c>
       <c r="D10" t="s">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="E10" t="s">
-        <v>55</v>
-      </c>
-      <c r="F10">
+        <v>67</v>
+      </c>
+      <c r="L10">
         <v>500</v>
       </c>
-      <c r="G10" t="s">
-        <v>18</v>
-      </c>
-      <c r="H10">
+      <c r="M10" t="s">
+        <v>30</v>
+      </c>
+      <c r="N10">
         <v>10</v>
       </c>
-      <c r="I10" t="s">
-        <v>56</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="K10">
+      <c r="O10" t="s">
+        <v>68</v>
+      </c>
+      <c r="P10" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q10">
         <v>5</v>
       </c>
-      <c r="L10">
+      <c r="R10">
         <v>4</v>
       </c>
-      <c r="M10">
+      <c r="S10">
         <v>3</v>
       </c>
-      <c r="N10">
+      <c r="T10">
         <v>2</v>
       </c>
-      <c r="O10">
+      <c r="U10">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:21">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="C11">
         <v>1111</v>
       </c>
       <c r="D11" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="E11" t="s">
-        <v>60</v>
-      </c>
-      <c r="F11">
+        <v>72</v>
+      </c>
+      <c r="L11">
         <v>500</v>
       </c>
-      <c r="G11" t="s">
-        <v>18</v>
-      </c>
-      <c r="H11">
+      <c r="M11" t="s">
+        <v>30</v>
+      </c>
+      <c r="N11">
         <v>11</v>
       </c>
-      <c r="I11" t="s">
-        <v>61</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="K11">
+      <c r="O11" t="s">
+        <v>73</v>
+      </c>
+      <c r="P11" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q11">
         <v>5</v>
       </c>
-      <c r="L11">
+      <c r="R11">
         <v>4</v>
       </c>
-      <c r="M11">
+      <c r="S11">
         <v>3</v>
       </c>
-      <c r="N11">
+      <c r="T11">
         <v>2</v>
       </c>
-      <c r="O11">
+      <c r="U11">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add packing request to product and cart
</commit_message>
<xml_diff>
--- a/Products.xlsx
+++ b/Products.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="76">
   <si>
     <t>id</t>
   </si>
@@ -76,6 +76,9 @@
     <t>size</t>
   </si>
   <si>
+    <t>packing</t>
+  </si>
+  <si>
     <t>Category</t>
   </si>
   <si>
@@ -125,6 +128,9 @@
   </si>
   <si>
     <t>1*1</t>
+  </si>
+  <si>
+    <t>COLOR_BOX</t>
   </si>
   <si>
     <t>Electronics</t>
@@ -1196,7 +1202,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:V11"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.1"/>
   <cols>
     <col min="1" max="1" width="14.6576576576577" customWidth="1"/>
@@ -1211,15 +1217,15 @@
     <col min="10" max="10" width="24.4324324324324" customWidth="1"/>
     <col min="11" max="11" width="28.2432432432432" customWidth="1"/>
     <col min="13" max="13" width="13.8918918918919" customWidth="1"/>
-    <col min="16" max="16" width="15.2612612612613" customWidth="1"/>
-    <col min="17" max="17" width="11.1711711711712" customWidth="1"/>
-    <col min="18" max="18" width="11.6216216216216" customWidth="1"/>
-    <col min="19" max="19" width="11.3513513513514" customWidth="1"/>
-    <col min="20" max="20" width="11.7117117117117" customWidth="1"/>
-    <col min="21" max="21" width="13.3513513513514" customWidth="1"/>
+    <col min="16" max="17" width="15.2612612612613" customWidth="1"/>
+    <col min="18" max="18" width="11.1711711711712" customWidth="1"/>
+    <col min="19" max="19" width="11.6216216216216" customWidth="1"/>
+    <col min="20" max="20" width="11.3513513513514" customWidth="1"/>
+    <col min="21" max="21" width="11.7117117117117" customWidth="1"/>
+    <col min="22" max="22" width="13.3513513513514" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21">
+    <row r="1" spans="1:22">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1283,492 +1289,507 @@
       <c r="U1" t="s">
         <v>20</v>
       </c>
+      <c r="V1" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="2" ht="14.15" spans="1:21">
+    <row r="2" ht="14.15" spans="1:22">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C2" s="2">
         <v>500</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L2">
         <v>500</v>
       </c>
       <c r="M2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N2">
         <v>2</v>
       </c>
       <c r="O2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q2">
+        <v>33</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="R2">
         <v>5</v>
       </c>
-      <c r="R2">
+      <c r="S2">
         <v>4</v>
       </c>
-      <c r="S2">
+      <c r="T2">
         <v>3</v>
       </c>
-      <c r="T2">
+      <c r="U2">
         <v>2</v>
       </c>
-      <c r="U2">
+      <c r="V2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" ht="14.15" spans="1:21">
+    <row r="3" ht="14.15" spans="1:22">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C3" s="2">
         <v>1000</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="L3">
         <v>500</v>
       </c>
       <c r="M3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N3">
         <v>3</v>
       </c>
       <c r="O3" t="s">
-        <v>36</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q3">
+        <v>38</v>
+      </c>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="R3">
         <v>5</v>
       </c>
-      <c r="R3">
+      <c r="S3">
         <v>4</v>
       </c>
-      <c r="S3">
+      <c r="T3">
         <v>3</v>
       </c>
-      <c r="T3">
+      <c r="U3">
         <v>2</v>
       </c>
-      <c r="U3">
+      <c r="V3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" ht="14.15" spans="1:21">
+    <row r="4" ht="14.15" spans="1:22">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C4" s="2">
         <v>520</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="L4">
         <v>500</v>
       </c>
       <c r="M4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N4">
         <v>4</v>
       </c>
       <c r="O4" t="s">
-        <v>40</v>
-      </c>
-      <c r="P4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q4">
+        <v>42</v>
+      </c>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="R4">
         <v>5</v>
       </c>
-      <c r="R4">
+      <c r="S4">
         <v>4</v>
       </c>
-      <c r="S4">
+      <c r="T4">
         <v>3</v>
       </c>
-      <c r="T4">
+      <c r="U4">
         <v>2</v>
       </c>
-      <c r="U4">
+      <c r="V4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" ht="14.15" spans="1:21">
+    <row r="5" ht="14.15" spans="1:22">
       <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C5" s="2">
         <v>1314</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L5">
         <v>500</v>
       </c>
       <c r="M5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N5">
         <v>5</v>
       </c>
       <c r="O5" t="s">
-        <v>44</v>
-      </c>
-      <c r="P5" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q5">
+        <v>46</v>
+      </c>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="R5">
         <v>5</v>
       </c>
-      <c r="R5">
+      <c r="S5">
         <v>4</v>
       </c>
-      <c r="S5">
+      <c r="T5">
         <v>3</v>
       </c>
-      <c r="T5">
+      <c r="U5">
         <v>2</v>
       </c>
-      <c r="U5">
+      <c r="V5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:21">
+    <row r="6" spans="1:22">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C6">
         <v>9999</v>
       </c>
       <c r="D6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L6">
         <v>500</v>
       </c>
       <c r="M6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N6">
         <v>6</v>
       </c>
       <c r="O6" t="s">
-        <v>48</v>
-      </c>
-      <c r="P6" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="Q6">
+        <v>50</v>
+      </c>
+      <c r="P6" s="3"/>
+      <c r="Q6" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="R6">
         <v>5</v>
       </c>
-      <c r="R6">
+      <c r="S6">
         <v>4</v>
       </c>
-      <c r="S6">
+      <c r="T6">
         <v>3</v>
       </c>
-      <c r="T6">
+      <c r="U6">
         <v>2</v>
       </c>
-      <c r="U6">
+      <c r="V6">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:21">
+    <row r="7" spans="1:22">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C7">
         <v>8888</v>
       </c>
       <c r="D7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="L7">
         <v>500</v>
       </c>
       <c r="M7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N7">
         <v>7</v>
       </c>
       <c r="O7" t="s">
-        <v>53</v>
-      </c>
-      <c r="P7" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="Q7">
+        <v>55</v>
+      </c>
+      <c r="P7" s="3"/>
+      <c r="Q7" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="R7">
         <v>5</v>
       </c>
-      <c r="R7">
+      <c r="S7">
         <v>4</v>
       </c>
-      <c r="S7">
+      <c r="T7">
         <v>3</v>
       </c>
-      <c r="T7">
+      <c r="U7">
         <v>2</v>
       </c>
-      <c r="U7">
+      <c r="V7">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:21">
+    <row r="8" spans="1:22">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C8">
         <v>6666</v>
       </c>
       <c r="D8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="L8">
         <v>500</v>
       </c>
       <c r="M8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N8">
         <v>8</v>
       </c>
       <c r="O8" t="s">
-        <v>58</v>
-      </c>
-      <c r="P8" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q8">
+        <v>60</v>
+      </c>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="R8">
         <v>5</v>
       </c>
-      <c r="R8">
+      <c r="S8">
         <v>4</v>
       </c>
-      <c r="S8">
+      <c r="T8">
         <v>3</v>
       </c>
-      <c r="T8">
+      <c r="U8">
         <v>2</v>
       </c>
-      <c r="U8">
+      <c r="V8">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:21">
+    <row r="9" spans="1:22">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C9">
         <v>4444</v>
       </c>
       <c r="D9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E9" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="L9">
         <v>500</v>
       </c>
       <c r="M9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N9">
         <v>9</v>
       </c>
       <c r="O9" t="s">
-        <v>63</v>
-      </c>
-      <c r="P9" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q9">
+        <v>65</v>
+      </c>
+      <c r="P9" s="3"/>
+      <c r="Q9" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="R9">
         <v>5</v>
       </c>
-      <c r="R9">
+      <c r="S9">
         <v>4</v>
       </c>
-      <c r="S9">
+      <c r="T9">
         <v>3</v>
       </c>
-      <c r="T9">
+      <c r="U9">
         <v>2</v>
       </c>
-      <c r="U9">
+      <c r="V9">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:21">
+    <row r="10" spans="1:22">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C10">
         <v>2222</v>
       </c>
       <c r="D10" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="L10">
         <v>500</v>
       </c>
       <c r="M10" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N10">
         <v>10</v>
       </c>
       <c r="O10" t="s">
-        <v>68</v>
-      </c>
-      <c r="P10" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q10">
+        <v>70</v>
+      </c>
+      <c r="P10" s="3"/>
+      <c r="Q10" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="R10">
         <v>5</v>
       </c>
-      <c r="R10">
+      <c r="S10">
         <v>4</v>
       </c>
-      <c r="S10">
+      <c r="T10">
         <v>3</v>
       </c>
-      <c r="T10">
+      <c r="U10">
         <v>2</v>
       </c>
-      <c r="U10">
+      <c r="V10">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:21">
+    <row r="11" spans="1:22">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C11">
         <v>1111</v>
       </c>
       <c r="D11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E11" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L11">
         <v>500</v>
       </c>
       <c r="M11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N11">
         <v>11</v>
       </c>
       <c r="O11" t="s">
-        <v>73</v>
-      </c>
-      <c r="P11" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="Q11">
+        <v>75</v>
+      </c>
+      <c r="P11" s="3"/>
+      <c r="Q11" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="R11">
         <v>5</v>
       </c>
-      <c r="R11">
+      <c r="S11">
         <v>4</v>
       </c>
-      <c r="S11">
+      <c r="T11">
         <v>3</v>
       </c>
-      <c r="T11">
+      <c r="U11">
         <v>2</v>
       </c>
-      <c r="U11">
+      <c r="V11">
         <v>1</v>
       </c>
     </row>

</xml_diff>